<commit_message>
update SW version 27 Aug 2026
</commit_message>
<xml_diff>
--- a/bug-tracker/UBA-bugs-tracker.xlsx
+++ b/bug-tracker/UBA-bugs-tracker.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work\DEV\UBA6-release\bug-tracker\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work\DEV\UBA6-maintenance\bug-tracker\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E45D976-C5D9-4015-B05A-A7EFFB0DCC42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A117F1C-0413-415F-B52B-9E6AEA6165E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{5B816FF3-3B79-4319-AB68-882518EDFCB6}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5B816FF3-3B79-4319-AB68-882518EDFCB6}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="99">
   <si>
     <t>Num</t>
   </si>
@@ -368,12 +368,18 @@
   <si>
     <t>הגדרת סדר הטסטים לא נכונה - תוקן</t>
   </si>
+  <si>
+    <t>tryAgagin</t>
+  </si>
+  <si>
+    <t>18.08.2026</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -448,6 +454,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="5"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -504,7 +518,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -583,6 +597,9 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1395,10 +1412,12 @@
       <c r="F17" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="G17" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="H17" s="6"/>
+      <c r="G17" s="30" t="s">
+        <v>97</v>
+      </c>
+      <c r="H17" s="8" t="s">
+        <v>98</v>
+      </c>
       <c r="I17" s="21" t="s">
         <v>55</v>
       </c>
@@ -1425,10 +1444,12 @@
       <c r="F18" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="G18" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="H18" s="6"/>
+      <c r="G18" s="30" t="s">
+        <v>97</v>
+      </c>
+      <c r="H18" s="8" t="s">
+        <v>98</v>
+      </c>
       <c r="I18" s="21" t="s">
         <v>56</v>
       </c>
@@ -1517,10 +1538,12 @@
       <c r="F21" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="G21" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="H21" s="6"/>
+      <c r="G21" s="30" t="s">
+        <v>97</v>
+      </c>
+      <c r="H21" s="8" t="s">
+        <v>98</v>
+      </c>
       <c r="I21" s="21" t="s">
         <v>55</v>
       </c>
@@ -1547,10 +1570,12 @@
       <c r="F22" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="G22" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="H22" s="6"/>
+      <c r="G22" s="30" t="s">
+        <v>97</v>
+      </c>
+      <c r="H22" s="8" t="s">
+        <v>98</v>
+      </c>
       <c r="I22" s="20"/>
       <c r="J22" s="5"/>
       <c r="K22" s="5"/>
@@ -1575,10 +1600,12 @@
       <c r="F23" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="G23" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="H23" s="6"/>
+      <c r="G23" s="30" t="s">
+        <v>97</v>
+      </c>
+      <c r="H23" s="8" t="s">
+        <v>98</v>
+      </c>
       <c r="I23" s="20"/>
       <c r="J23" s="5"/>
       <c r="K23" s="5"/>
@@ -1603,8 +1630,8 @@
       <c r="F24" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="G24" s="10" t="s">
-        <v>18</v>
+      <c r="G24" s="9" t="s">
+        <v>11</v>
       </c>
       <c r="H24" s="6"/>
       <c r="I24" s="22"/>
@@ -1733,10 +1760,12 @@
       <c r="F28" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="G28" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="H28" s="6"/>
+      <c r="G28" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="H28" s="8" t="s">
+        <v>98</v>
+      </c>
       <c r="I28" s="20"/>
       <c r="J28" s="5"/>
       <c r="K28" s="5"/>

</xml_diff>